<commit_message>
Llena datos del grupo en la hoja Instrucciones del Excel de entrega 1
</commit_message>
<xml_diff>
--- a/cerebro-londres/Diccionario_de_datos_TallerDatos.xlsx
+++ b/cerebro-londres/Diccionario_de_datos_TallerDatos.xlsx
@@ -574,21 +574,21 @@
     <row r="5">
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Ciudad elegida:</t>
+          <t>Ciudad elegida: Londres</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Integrantes:</t>
+          <t>Integrantes: Jean Carlo Ardila - David Cossio - Juan Pablo Posso</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Enlace al repositorio o a la carpeta del lago:</t>
+          <t>Enlace al repositorio o a la carpeta del lago: https://github.com/JeanArdila711/cerebro-londres</t>
         </is>
       </c>
     </row>

</xml_diff>